<commit_message>
Registro CORPOGESTAR GHV567 20260420_194849
</commit_message>
<xml_diff>
--- a/database.xlsx
+++ b/database.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J37"/>
+  <dimension ref="A1:J40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2266,6 +2266,156 @@
       <c r="J37" t="inlineStr">
         <is>
           <t>Sin foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>80</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>40</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>120</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
         </is>
       </c>
     </row>
@@ -2280,7 +2430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2985,6 +3135,156 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
+        <v>80</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G16" t="n">
+        <v>40</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>April_2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>CORPOGESTAR</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Fabián</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>GHV567</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Cartón limpio</t>
+        </is>
+      </c>
+      <c r="G17" t="n">
+        <v>120</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>No hubo observaciones</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/MEMO_20260420_194849.jpg</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/alejandraho013/registro-salida-residuos/main/fotos/CAMION_20260420_194849.jpg</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>